<commit_message>
Migrate AA flow IDs to typed naming
</commit_message>
<xml_diff>
--- a/aa/xlsx/event-logging-map.xlsx
+++ b/aa/xlsx/event-logging-map.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>IF-006</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>IF-006</t>
+          <t>L0</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -832,12 +832,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Исключение Labels API: path, statusCode, safe message</t>
+          <t>Исключение обработчика Labels API: path, statusCode, safe message</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>HTTP status / текст ошибки</t>
+          <t>Текст ошибки</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">

</xml_diff>